<commit_message>
juntei a bspd em 1 unico ficheiro
</commit_message>
<xml_diff>
--- a/Simbolos/Componentes.xlsx
+++ b/Simbolos/Componentes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AA\Desktop\faculdade (Pasta nova)\Mestrado\Formula Student\Coisa Qspice\Qspice-Library\Simbolos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25ABAD0F-0EE3-453B-BD61-6A9B768F0739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F084EAE5-62C6-4808-88F2-68FAC8DC3DDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{1AEE4442-FBE4-43B0-AA6E-ACCDBFA4DCB0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{1AEE4442-FBE4-43B0-AA6E-ACCDBFA4DCB0}"/>
   </bookViews>
   <sheets>
     <sheet name="Comparadores" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="46">
   <si>
     <t>Canais</t>
   </si>
@@ -170,13 +170,19 @@
   </si>
   <si>
     <t>H (Ganho Min-Max)</t>
+  </si>
+  <si>
+    <t>Simula limites do componente</t>
+  </si>
+  <si>
+    <t>não</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -203,13 +209,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -236,10 +254,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
@@ -247,8 +266,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Bad" xfId="1" builtinId="27"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -581,23 +604,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE87AEAF-12FF-46B3-81D1-C75236B9FFDD}">
-  <dimension ref="B2:M11"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="B2:N11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="16.625" customWidth="1"/>
-    <col min="4" max="4" width="9.875" customWidth="1"/>
-    <col min="5" max="7" width="10.125" customWidth="1"/>
-    <col min="8" max="8" width="14.625" customWidth="1"/>
-    <col min="9" max="9" width="14.75" customWidth="1"/>
-    <col min="10" max="10" width="14.875" customWidth="1"/>
-    <col min="11" max="11" width="14.5" customWidth="1"/>
-    <col min="12" max="12" width="14.625" customWidth="1"/>
-    <col min="13" max="13" width="16.375" customWidth="1"/>
+    <col min="2" max="3" width="16.5703125" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" customWidth="1"/>
+    <col min="5" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" customWidth="1"/>
+    <col min="10" max="10" width="14.85546875" customWidth="1"/>
+    <col min="11" max="11" width="14.42578125" customWidth="1"/>
+    <col min="12" max="12" width="14.5703125" customWidth="1"/>
+    <col min="13" max="13" width="16.42578125" customWidth="1"/>
     <col min="18" max="18" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" ht="15" thickBot="1"/>
-    <row r="3" spans="2:13" ht="30.75" thickBot="1">
+    <row r="2" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:14" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
@@ -634,8 +657,11 @@
       <c r="M3" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="2:13" ht="15.75" thickBot="1">
+      <c r="N3" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="2:14" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>12</v>
       </c>
@@ -670,8 +696,11 @@
         <v>9</v>
       </c>
       <c r="M4" s="2"/>
-    </row>
-    <row r="5" spans="2:13" ht="15.75" thickBot="1">
+      <c r="N4" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="2"/>
@@ -684,8 +713,9 @@
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
-    </row>
-    <row r="6" spans="2:13" ht="15.75" thickBot="1">
+      <c r="N5" s="2"/>
+    </row>
+    <row r="6" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="2"/>
@@ -698,8 +728,9 @@
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
-    </row>
-    <row r="7" spans="2:13" ht="15.75" thickBot="1">
+      <c r="N6" s="2"/>
+    </row>
+    <row r="7" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="2"/>
@@ -712,8 +743,9 @@
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
-    </row>
-    <row r="8" spans="2:13" ht="15.75" thickBot="1">
+      <c r="N7" s="2"/>
+    </row>
+    <row r="8" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="2"/>
@@ -726,8 +758,9 @@
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
-    </row>
-    <row r="9" spans="2:13" ht="15.75" thickBot="1">
+      <c r="N8" s="2"/>
+    </row>
+    <row r="9" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="2"/>
@@ -740,8 +773,9 @@
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
-    </row>
-    <row r="10" spans="2:13" ht="15.75" thickBot="1">
+      <c r="N9" s="2"/>
+    </row>
+    <row r="10" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="2"/>
@@ -754,8 +788,9 @@
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
-    </row>
-    <row r="11" spans="2:13" ht="15.75" thickBot="1">
+      <c r="N10" s="2"/>
+    </row>
+    <row r="11" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="2"/>
@@ -768,6 +803,7 @@
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -778,17 +814,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D09A1AF3-FAAD-437D-B280-69CCB64B857F}">
-  <dimension ref="B1:J5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="B1:K4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="16.375" customWidth="1"/>
-    <col min="6" max="6" width="16.5" customWidth="1"/>
-    <col min="7" max="7" width="15.25" customWidth="1"/>
-    <col min="9" max="10" width="18.5" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" customWidth="1"/>
+    <col min="10" max="10" width="18.42578125" customWidth="1"/>
+    <col min="11" max="11" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" thickBot="1"/>
-    <row r="2" spans="2:10" ht="45.75" thickBot="1">
+    <row r="1" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:11" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
@@ -816,8 +854,11 @@
       <c r="J2" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="3" spans="2:10" ht="30.75" thickBot="1">
+      <c r="K2" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>38</v>
       </c>
@@ -843,8 +884,11 @@
         <v>42</v>
       </c>
       <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="2:10" ht="15.75" thickBot="1">
+      <c r="K3" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -854,8 +898,8 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="2:10" ht="14.25"/>
+      <c r="K4" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -863,21 +907,22 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{302B899F-8279-44A8-AE92-7781FBA7A931}">
-  <dimension ref="B1:K6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="B1:L5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.375" customWidth="1"/>
-    <col min="2" max="2" width="15.875" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
-    <col min="6" max="6" width="20.375" customWidth="1"/>
-    <col min="7" max="7" width="16.625" customWidth="1"/>
+    <col min="6" max="6" width="20.42578125" customWidth="1"/>
+    <col min="7" max="7" width="16.5703125" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="19.25" customWidth="1"/>
-    <col min="10" max="10" width="16.75" customWidth="1"/>
+    <col min="9" max="9" width="19.28515625" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" customWidth="1"/>
+    <col min="12" max="12" width="23.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" thickBot="1"/>
-    <row r="2" spans="2:11" ht="15.75" thickBot="1">
+    <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:12" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
@@ -908,8 +953,11 @@
       <c r="K2" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="3" spans="2:11" ht="15.75" thickBot="1">
+      <c r="L2" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>18</v>
       </c>
@@ -938,8 +986,11 @@
         <v>0.5</v>
       </c>
       <c r="K3" s="2"/>
-    </row>
-    <row r="4" spans="2:11" ht="15.75" thickBot="1">
+      <c r="L3" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>20</v>
       </c>
@@ -969,8 +1020,9 @@
         <v>0.5</v>
       </c>
       <c r="K4" s="2"/>
-    </row>
-    <row r="5" spans="2:11" ht="15.75" thickBot="1">
+      <c r="L4" s="2"/>
+    </row>
+    <row r="5" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -981,8 +1033,8 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
-    </row>
-    <row r="6" spans="2:11" ht="14.25"/>
+      <c r="L5" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>